<commit_message>
Update data files and scripts - 2026-03-15
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/nifty_options/nifty_options_2026-03.xlsx
+++ b/data/nifty_options/nifty_options_2026-03.xlsx
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE2"/>
+  <dimension ref="A1:AE8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -788,6 +788,708 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-04</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>10:00:13</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>TRADEABLE</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="6" t="n">
+        <v>24325.3</v>
+      </c>
+      <c r="I3" s="6" t="n">
+        <v>20.79</v>
+      </c>
+      <c r="J3" s="6" t="n">
+        <v>7.73</v>
+      </c>
+      <c r="K3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="5" t="n">
+        <v>98.09999999999999</v>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="N3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3" s="2" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="U3" s="2" t="inlineStr"/>
+      <c r="V3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC3" s="2" t="inlineStr">
+        <is>
+          <t>HARD VETO: CPR TRENDING DAY: Price 24325.30 below BC 24796.42 - BEARISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AD3" s="2" t="inlineStr">
+        <is>
+          <t>CPR TRENDING DAY: Price 24325.30 below BC 24796.42 - BEARISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AE3" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>10:00:10</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>TRADEABLE</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="6" t="n">
+        <v>23774</v>
+      </c>
+      <c r="I4" s="6" t="n">
+        <v>24.25</v>
+      </c>
+      <c r="J4" s="6" t="n">
+        <v>3.11</v>
+      </c>
+      <c r="K4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="5" t="n">
+        <v>99.59999999999999</v>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="N4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4" s="2" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="U4" s="2" t="inlineStr"/>
+      <c r="V4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC4" s="2" t="inlineStr">
+        <is>
+          <t>HARD VETO: CPR TRENDING DAY: Price 23774.00 below BC 24558.28 - BEARISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AD4" s="2" t="inlineStr">
+        <is>
+          <t>CPR TRENDING DAY: Price 23774.00 below BC 24558.28 - BEARISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AE4" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>10:00:13</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>TRADEABLE</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>24092.45</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>20.81</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="K5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="5" t="n">
+        <v>97.40000000000001</v>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="N5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" s="2" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="U5" s="2" t="inlineStr"/>
+      <c r="V5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC5" s="2" t="inlineStr">
+        <is>
+          <t>HARD VETO: CPR TRENDING DAY: Price 24092.45 above TC 23981.36 - BULLISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AD5" s="2" t="inlineStr">
+        <is>
+          <t>CPR TRENDING DAY: Price 24092.45 above TC 23981.36 - BULLISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>10:00:12</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>TRADEABLE</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>24151.85</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>19.27</v>
+      </c>
+      <c r="J6" s="6" t="n">
+        <v>-0.61</v>
+      </c>
+      <c r="K6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="5" t="n">
+        <v>96.59999999999999</v>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="N6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T6" s="2" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="U6" s="2" t="inlineStr"/>
+      <c r="V6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC6" s="2" t="inlineStr">
+        <is>
+          <t>HARD VETO: CPR TRENDING DAY: Price 24151.85 below BC 24191.88 - BEARISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AD6" s="2" t="inlineStr">
+        <is>
+          <t>CPR TRENDING DAY: Price 24151.85 below BC 24191.88 - BEARISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AE6" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-12</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>10:00:08</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>TRADEABLE</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>23695.3</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>21.99</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>-1.37</v>
+      </c>
+      <c r="K7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="5" t="n">
+        <v>98.90000000000001</v>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="N7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" s="2" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="U7" s="2" t="inlineStr"/>
+      <c r="V7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB7" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC7" s="2" t="inlineStr">
+        <is>
+          <t>HARD VETO: CPR TRENDING DAY: Price 23695.30 below BC 24066.65 - BEARISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AD7" s="2" t="inlineStr">
+        <is>
+          <t>CPR TRENDING DAY: Price 23695.30 below BC 24066.65 - BEARISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AE7" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>10:00:17</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>TRADEABLE</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>23348.85</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>21.83</v>
+      </c>
+      <c r="J8" s="6" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="K8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="5" t="n">
+        <v>98.90000000000001</v>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T8" s="2" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="U8" s="2" t="inlineStr"/>
+      <c r="V8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC8" s="2" t="inlineStr">
+        <is>
+          <t>HARD VETO: CPR TRENDING DAY: Price 23348.85 below BC 23694.72 - BEARISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AD8" s="2" t="inlineStr">
+        <is>
+          <t>CPR TRENDING DAY: Price 23348.85 below BC 23694.72 - BEARISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AE8" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update data files and scripts - 2026-03-24
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/nifty_options/nifty_options_2026-03.xlsx
+++ b/data/nifty_options/nifty_options_2026-03.xlsx
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE8"/>
+  <dimension ref="A1:AE14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1490,6 +1490,708 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>10:00:17</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>TRADEABLE</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>23171.2</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>22.11</v>
+      </c>
+      <c r="J9" s="6" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="K9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="5" t="n">
+        <v>98.5</v>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="N9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T9" s="2" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="U9" s="2" t="inlineStr"/>
+      <c r="V9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB9" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC9" s="2" t="inlineStr">
+        <is>
+          <t>HARD VETO: CPR TRENDING DAY: Price 23171.20 below BC 23302.20 - BEARISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AD9" s="2" t="inlineStr">
+        <is>
+          <t>CPR TRENDING DAY: Price 23171.20 below BC 23302.20 - BEARISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AE9" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>10:00:18</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>TRADEABLE</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>23497.2</v>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>20.48</v>
+      </c>
+      <c r="J10" s="6" t="n">
+        <v>-1.04</v>
+      </c>
+      <c r="K10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="5" t="n">
+        <v>95.90000000000001</v>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="N10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T10" s="2" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="U10" s="2" t="inlineStr"/>
+      <c r="V10" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y10" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB10" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC10" s="2" t="inlineStr">
+        <is>
+          <t>HARD VETO: Market trending with avg daily range 1.55% &gt; 1.5% threshold - Bad for straddle selling</t>
+        </is>
+      </c>
+      <c r="AD10" s="2" t="inlineStr">
+        <is>
+          <t>Market trending with avg daily range 1.55% &gt; 1.5% threshold - Bad for straddle selling</t>
+        </is>
+      </c>
+      <c r="AE10" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>10:00:19</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>TRADEABLE</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>23693.9</v>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>18.95</v>
+      </c>
+      <c r="J11" s="6" t="n">
+        <v>-3.7</v>
+      </c>
+      <c r="K11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="5" t="n">
+        <v>93.7</v>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="N11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T11" s="2" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="U11" s="2" t="inlineStr"/>
+      <c r="V11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB11" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC11" s="2" t="inlineStr">
+        <is>
+          <t>HARD VETO: CPR TRENDING DAY: Price 23693.90 above TC 23554.67 - BULLISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AD11" s="2" t="inlineStr">
+        <is>
+          <t>CPR TRENDING DAY: Price 23693.90 above TC 23554.67 - BULLISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AE11" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>10:00:50</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>TRADEABLE</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>23236.75</v>
+      </c>
+      <c r="I12" s="6" t="n">
+        <v>21.64</v>
+      </c>
+      <c r="J12" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="K12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="5" t="n">
+        <v>98.5</v>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="N12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T12" s="2" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="U12" s="2" t="inlineStr"/>
+      <c r="V12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y12" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB12" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC12" s="2" t="inlineStr">
+        <is>
+          <t>HARD VETO: CPR TRENDING DAY: Price 23236.75 below BC 23740.35 - BEARISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AD12" s="2" t="inlineStr">
+        <is>
+          <t>CPR TRENDING DAY: Price 23236.75 below BC 23740.35 - BEARISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AE12" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>10:00:28</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>TRADEABLE</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="6" t="n">
+        <v>23260.05</v>
+      </c>
+      <c r="I13" s="6" t="n">
+        <v>22.26</v>
+      </c>
+      <c r="J13" s="6" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="K13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="5" t="n">
+        <v>98.5</v>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="N13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T13" s="2" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="U13" s="2" t="inlineStr"/>
+      <c r="V13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB13" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC13" s="2" t="inlineStr">
+        <is>
+          <t>HARD VETO: Market trending with avg daily range 1.51% &gt; 1.5% threshold - Bad for straddle selling</t>
+        </is>
+      </c>
+      <c r="AD13" s="2" t="inlineStr">
+        <is>
+          <t>Market trending with avg daily range 1.51% &gt; 1.5% threshold - Bad for straddle selling</t>
+        </is>
+      </c>
+      <c r="AE13" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-23</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>10:00:27</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>TRADEABLE</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>22598.4</v>
+      </c>
+      <c r="I14" s="6" t="n">
+        <v>26.11</v>
+      </c>
+      <c r="J14" s="6" t="n">
+        <v>7.39</v>
+      </c>
+      <c r="K14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="5" t="n">
+        <v>99.59999999999999</v>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="N14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" s="2" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="U14" s="2" t="inlineStr"/>
+      <c r="V14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC14" s="2" t="inlineStr">
+        <is>
+          <t>HARD VETO: CPR TRENDING DAY: Price 22598.40 below BC 23206.38 - BEARISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AD14" s="2" t="inlineStr">
+        <is>
+          <t>CPR TRENDING DAY: Price 22598.40 below BC 23206.38 - BEARISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AE14" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update data files and scripts - 2026-04-27
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/nifty_options/nifty_options_2026-03.xlsx
+++ b/data/nifty_options/nifty_options_2026-03.xlsx
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE14"/>
+  <dimension ref="A1:AE18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2192,6 +2192,474 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>10:00:28</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>TRADEABLE</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="6" t="n">
+        <v>22755.5</v>
+      </c>
+      <c r="I15" s="6" t="n">
+        <v>25.35</v>
+      </c>
+      <c r="J15" s="6" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="K15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="5" t="n">
+        <v>99.3</v>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="N15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T15" s="2" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="U15" s="2" t="inlineStr"/>
+      <c r="V15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC15" s="2" t="inlineStr">
+        <is>
+          <t>HARD VETO: CPR TRENDING DAY: Price 22755.50 above TC 22562.26 - BULLISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AD15" s="2" t="inlineStr">
+        <is>
+          <t>CPR TRENDING DAY: Price 22755.50 above TC 22562.26 - BULLISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AE15" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>10:00:20</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>TRADEABLE</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="6" t="n">
+        <v>23286.85</v>
+      </c>
+      <c r="I16" s="6" t="n">
+        <v>24.64</v>
+      </c>
+      <c r="J16" s="6" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="K16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="5" t="n">
+        <v>98.90000000000001</v>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="N16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T16" s="2" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="U16" s="2" t="inlineStr"/>
+      <c r="V16" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB16" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC16" s="2" t="inlineStr">
+        <is>
+          <t>HARD VETO: Market trending with avg daily range 1.55% &gt; 1.5% threshold - Bad for straddle selling</t>
+        </is>
+      </c>
+      <c r="AD16" s="2" t="inlineStr">
+        <is>
+          <t>Market trending with avg daily range 1.55% &gt; 1.5% threshold - Bad for straddle selling</t>
+        </is>
+      </c>
+      <c r="AE16" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-27</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>10:00:18</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>TRADEABLE</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="6" t="n">
+        <v>22991.85</v>
+      </c>
+      <c r="I17" s="6" t="n">
+        <v>26.91</v>
+      </c>
+      <c r="J17" s="6" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="K17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="5" t="n">
+        <v>99.59999999999999</v>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="N17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T17" s="2" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="U17" s="2" t="inlineStr"/>
+      <c r="V17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y17" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA17" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB17" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC17" s="2" t="inlineStr">
+        <is>
+          <t>HARD VETO: CPR TRENDING DAY: Price 22991.85 below BC 23264.28 - BEARISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AD17" s="2" t="inlineStr">
+        <is>
+          <t>CPR TRENDING DAY: Price 22991.85 below BC 23264.28 - BEARISH TRENDING DAY likely</t>
+        </is>
+      </c>
+      <c r="AE17" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>10:00:21</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>AVOID</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>TRADEABLE</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="6" t="n">
+        <v>22613.9</v>
+      </c>
+      <c r="I18" s="6" t="n">
+        <v>28.33</v>
+      </c>
+      <c r="J18" s="6" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="K18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="N18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T18" s="2" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="U18" s="2" t="inlineStr"/>
+      <c r="V18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="X18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA18" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB18" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC18" s="2" t="inlineStr">
+        <is>
+          <t>HARD VETO: Market trending with avg daily range 1.61% &gt; 1.5% threshold - Bad for straddle selling</t>
+        </is>
+      </c>
+      <c r="AD18" s="2" t="inlineStr">
+        <is>
+          <t>Market trending with avg daily range 1.61% &gt; 1.5% threshold - Bad for straddle selling</t>
+        </is>
+      </c>
+      <c r="AE18" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>